<commit_message>
docs(seo): add Google Trends and SERP results to keyword sheet
Trends: 21 keywords en España, grupos de 5 términos (medias solo comparables dentro del grupo).
SERP: resultado dominante por keyword en Google.es (gl=es, hl=es), 19/10/2026.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBD2ubJqcRcA9NTshfMy45
</commit_message>
<xml_diff>
--- a/research_notes/keywords/KEYWORD_RESEARCH_LANDING.xlsx
+++ b/research_notes/keywords/KEYWORD_RESEARCH_LANDING.xlsx
@@ -553,12 +553,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 69 (grupo A, 5 términos). Pico 100 (9 nov 2025), mínimo 44 (ago 2026), 62 al 18/10/2026. Alta y estable</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Marca de OpenAI (chatgpt.com) y ChatGPT.com/help; sin hueco para contenido</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Término de marca de tercero con volumen masivo. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Término de marca de tercero con volumen masivo. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -612,12 +612,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 32 (grupo A). Subida fuerte: de 19 a 52 en el año; 51 al 18/10/2026</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Google Gemini (gemini.google.com) y Google; sin hueco</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Término de marca de tercero. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Término de marca de tercero. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -671,12 +671,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 1 (grupo A). Muy bajo frente a chatgpt, con picos puntuales</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>chatgpt.com (plan gratis) y guías; intención de gratuidad</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Intención de gratuidad; no compite con afiliación. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Intención de gratuidad; no compite con afiliación. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -730,12 +730,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 0 (grupo A). Casi nula en esta escala; consultas en ascenso: grok, midjourney</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Herramientas (ChatGPT, Canva, Adobe Firefly, Meta AI, Bing): comparativa de herramientas</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Comparativa de herramientas con intención comercial. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Comparativa de herramientas con intención comercial. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -789,12 +789,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 18 (grupo B). Estable en 20-24 hasta julio 2026; 10 al 18/10/2026</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Guías informacionales y generadores de prompts (Jotform, Xataka, Cyberclick, UNIR, PromptsEra)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Encaja con el modelo de packs ASPECCT (ver modelo de negocio del handoff). Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Encaja con el modelo de packs ASPECCT (ver modelo de negocio del handoff). Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -848,12 +848,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 0-1 (grupo A). Casi nula en esta escala; pico puntual de consultas 'curso claude', 'claude cowork'</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>claude.ai (marca) y listados de modelos; sin hueco para contenido de terceros</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Término de marca de tercero. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Término de marca de tercero. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -907,12 +907,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 65 (grupo B). Pico 100 (feb 2026); 25 al 18/10/2026: caída fuerte</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>WordPress.com (oficial), Wikipedia y guías de creación; mixto marca/informacional</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Término muy amplio; mejor como clúster de comparativas. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Término muy amplio; mejor como clúster de comparativas. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -966,12 +966,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 7 (grupo B). Estable y baja; 4 al 18/10/2026</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>framer.com (oficial) y guías; nicho pequeño</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Comparativa de constructores web. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Comparativa de constructores web. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1025,12 +1025,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 6 (grupo B). Estable y baja; 4 al 18/10/2026</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>zapier.com (oficial), Wikipedia y guías en vídeo; intención de herramienta</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Encaja con el clúster no-code del modelo de negocio. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Encaja con el clúster no-code del modelo de negocio. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1084,12 +1084,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 28 (grupo B). Pico 49 (nov 2025); 9 al 18/10/2026: caída fuerte</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>n8n.io (oficial), Xataka, OpenWebinars, Wikipedia, NocodeHackers; guías y oficial</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Encaja con automatización de IA. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Encaja con automatización de IA. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1143,12 +1143,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 14 (grupo C). Pico 34 (mar 2026); 5 al 18/10/2026</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>semrush.com (oficial) y guías de SEO</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Término de marca de tercero con intención comercial. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Término de marca de tercero con intención comercial. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1206,12 +1206,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 2 (grupo C). Casi nula en esta escala; consulta en ascenso: 'best keyword research tools' (+90 %)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Blog de Semrush, IEBS, Marketing4eCommerce ('+10 herramientas'), Keyword Tool; guías y listados de herramientas: encaja con comparativas</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Puja alta observada; ver reports/Servicios digitales España.md. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Puja alta observada; ver reports/Servicios digitales España.md. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1269,12 +1269,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 6 (grupo C). 2 al 18/10/2026</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>ahrefs.com (oficial), tutoriales y guías; marca</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Puja alta observada; término de marca. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Puja alta observada; término de marca. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1332,12 +1332,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 5 (grupo C). 3 al 18/10/2026</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Google for Developers (guía), Wikipedia y map pack de agencias de Barcelona: mixto local/guía</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Puja más alta observada del clúster SEO. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Puja más alta observada del clúster SEO. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1391,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 79 (grupo C). Pico 100 (15 mar 2026); 67 al 18/10/2026</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>notion.com (oficial) y guías; marca de tercero</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Término de marca de tercero con volumen alto. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Término de marca de tercero con volumen alto. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1450,12 +1450,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 10 (grupo C). Picos por noticias de aplazamiento (100 el 30/11/2025; 37 el 4/10/2026 y 20 el 18/10/2026). Dirigida por eventos</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Agencia Tributaria (oficial), noticias de aplazamiento y software (verifactu.com, Cegid, Wolters Kluwer, Contasimple, Holded): informacional y noticias</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Tema regulatorio español; posible contenido de actualidad. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Tema regulatorio español; posible contenido de actualidad. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1509,12 +1509,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 16 (grupo D). Estable entre 15-20; 8 al 18/10/2026</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Salesforce, Wikipedia, HubSpot, Zoho, Oracle, Microsoft: guías de fabricantes</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Término amplio; mejor como clúster. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Término amplio; mejor como clúster. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1568,12 +1568,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 1 (grupo D). Casi nula; consultas no relacionadas (vuelos, viajes)</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Creatio, SoftDoit (comparativa de 190 soluciones), HubSpot, Salesforce, Recursos para Pymes ('16 mejores CRM gratis'): comparativas</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Intención comercial más clara que 'crm'. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Intención comercial más clara que 'crm'. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1627,12 +1627,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 4 (grupo D). Estable y baja</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Mailchimp, Brevo, Wikipedia, IEBS ('15 mejores herramientas'), Doppler, Mailrelay: guías y listados</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>Intención comercial; mucha competencia de SaaS. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Intención comercial; mucha competencia de SaaS. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1686,12 +1686,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 2 (grupo A). Baja y estable</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Constructores de web (Canva, IONOS, Wix, GoDaddy, Squarespace) y anuncios de agencias (189 €, 590 €, 899 €)</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>Keyword ya listada en el handoff; sin Trends ni SERP en esta hoja. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Keyword ya listada en el handoff; sin Trends ni SERP en esta hoja. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1745,12 +1745,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Media 70 (grupo A) y 12 (grupo D); grupos distintos. Pico 84 (mar 2026); 26 al 18/10/2026</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>No medido</t>
+          <t>Proveedores de hosting (Hostinger, IONOS, cdmon, OVHcloud, Arsys, SiteGround) en orgánico y anuncios</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Afiliación alta, pero la SERP está dominada por proveedores de hosting. Fuente: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
+          <t>Afiliación alta, pero la SERP está dominada por proveedores de hosting. Trends y SERP: Google Trends y Google.es (gl=es, hl=es), 19/10/2026. Fuente volumen: Google Ads Keyword Planner (España, español, red Google, oct 2025-sep 2026). Rango observado, no volumen exacto. Dato registrado en la sesión de transferencia (CLAUDE_HANDOFF.md)</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Medir las 21 keywords en España (mismo periodo) en grupos de 5 términos y registrar tendencia.</t>
+          <t>Hecho: 21 keywords en grupos de 5 términos (España, 12 meses). Las medias solo son comparables dentro de cada grupo (A-D).</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Revisar la SERP de las keywords con prioridad Alta: tipo de resultado, competidores y preguntas relacionadas.</t>
+          <t>Hecho: SERP de las 21 keywords en Google.es (resumen de resultados orgánicos dominantes).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
KW research: método gratuito de términos (21 keywords)
Hoja 'Términos (método gratis)' en el Excel con páginas válidas,
términos de consenso y especialistas por keyword. JSON de cada
keyword en research_notes/keywords/terminos/.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBD2ubJqcRcA9NTshfMy45
</commit_message>
<xml_diff>
--- a/research_notes/keywords/KEYWORD_RESEARCH_LANDING.xlsx
+++ b/research_notes/keywords/KEYWORD_RESEARCH_LANDING.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leyenda y pendientes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Términos (método gratis)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Keywords'!$A$1:$M$22</definedName>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +36,9 @@
     <font>
       <b val="1"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -62,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -73,6 +77,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1948,4 +1953,779 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Páginas válidas</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Páginas descartadas</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Cumple mínimo 10</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Nº términos consenso</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Top 10 consenso (tras filtro de números y repeticiones)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Nº términos especialistas</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt, datos, uso, puede, cómo, tiempo, son, cliente, openai, chat</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>google, gemini, artificial, inteligencia, inteligencia artificial, gemini puede, puede, modelos, cómo, usuarios</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 8 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>chatgpt gratis</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>No ejecutado: keyword sin lista de URLs. Pendiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>generador de imágenes ia</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>199</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>imagen, mejor, modelos, herramientas, uso, texto, calidad, generar, gratuito, contenido</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 8 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>prompts</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>prompts, chatgpt, prompt, datos, modelo, texto, mejores, claude, ejemplos, respuesta</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 8 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>claude ia</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>claude, anthropic, modelos, modelo, uso, tareas, cómo, pro, contexto, información</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 6 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>wordpress</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>wordpress, web, sitio, sitio web, crear, cómo, wordpress cómo, página, plugins, puede</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>framer</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>framer, code, page, basic, wordpress, drop, review, design, framer review, cms</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 5 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>zapier</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>zapier, make, visual, code, workflows, has, integromat, zapier make, apps, zaps</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 7 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>n8n</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>n8n, datos, flujo, trabajo, automatización, nodos, código, nodo, flujos, crear</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 6 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>semrush</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>semrush, software, opiniones, semrush seo, seo, mostrar, detalles, mostrar detalles, detalles semrush, marketing</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 6 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>keyword research</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>google, seo, ideas, marketing, keyword, web, solo, youtube, clave, palabras</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 9 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ahrefs</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>161</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>ahrefs, seo, clave, palabras, palabras clave, datos, herramientas, herramientas seo, web, backlinks</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 7 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>posicionamiento seo</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>116</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>seo, google, web, search, clave, contenido, búsqueda, resultados, cómo, página</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>notion</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>notion, datos, trabajo, tareas, base, proyectos, todo, puede, cómo, gestión</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 6 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>verifactu</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>182</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>verifactu, facturas, facturación, factura, empresas, autónomos, empresas autónomos, ley, electrónica, tributaria</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 9 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>crm</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>crm, clientes, cliente, ventas, gestión, marketing, empresa, empresas, puede, está</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>software crm</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>crm, clientes, ventas, marketing, empresa, mejor, software, cliente, empresas, herramientas</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>email marketing</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>marketing, email, email marketing, herramientas, emails, herramienta, campañas, contactos, también, empresas</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Muestra insuficiente: 6 páginas válidas (mínimo 10). Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>crear página web</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>web, sitio, crear, dominio, paso, tener, son, hacer, com, opciones</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>hosting</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>hosting, web, mejor, dominio, seguridad, planes, servicios, recursos, almacenamiento, son</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Ningún término especialista con este tamaño de muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Método: autocompletado y búsquedas reales de Google (es), páginas descargadas con curl y texto principal extraído; stopwords sin marca ni navegación. Consenso: cobertura ≥ 0,7. Especialista: cobertura ≤ 0,2 y frecuencia ≥ 5. Muestra por debajo de 10 páginas en la mayoría de keywords; resultados orientativos.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>